<commit_message>
push new stuff boiii
</commit_message>
<xml_diff>
--- a/schedule_output.xlsx
+++ b/schedule_output.xlsx
@@ -506,56 +506,52 @@
         </is>
       </c>
       <c r="B2" t="inlineStr"/>
-      <c r="C2" t="inlineStr"/>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>J17</t>
+        </is>
+      </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>J6, J17, J25</t>
+          <t>J2, J18, J26</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>J18</t>
+          <t>J5, J13</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
+          <t>J10, J23</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>J3, J14</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>J4, J24</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>J8, J12, J25</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr"/>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>J15, J21</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr"/>
+      <c r="N2" t="inlineStr">
+        <is>
           <t>J22</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>J8, J19, J21</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>J20</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>J26</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>J14</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>J23</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>J4</t>
-        </is>
-      </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>J11, J24</t>
         </is>
       </c>
       <c r="O2" t="inlineStr"/>
@@ -570,45 +566,45 @@
       <c r="B3" t="inlineStr"/>
       <c r="C3" t="inlineStr">
         <is>
-          <t>J1, J5</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
+          <t>J1</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr">
         <is>
           <t>J9</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>J2, J10, J13</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr"/>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>J6</t>
+        </is>
+      </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>J7</t>
+          <t>J19</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>J3</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr"/>
+          <t>J20</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>J7, J11</t>
+        </is>
+      </c>
       <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr"/>
       <c r="L3" t="inlineStr"/>
-      <c r="M3" t="inlineStr"/>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>J15</t>
-        </is>
-      </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>J12, J16</t>
-        </is>
-      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>J16</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr"/>
+      <c r="O3" t="inlineStr"/>
       <c r="P3" t="inlineStr"/>
     </row>
   </sheetData>
@@ -695,11 +691,11 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>L2</t>
+          <t>L1</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4">
@@ -720,11 +716,11 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>L2</t>
+          <t>L1</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="5">
@@ -749,7 +745,7 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>11</v>
+        <v>6</v>
       </c>
     </row>
     <row r="6">
@@ -770,11 +766,11 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>L2</t>
+          <t>L1</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="7">
@@ -795,11 +791,11 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>L1</t>
+          <t>L2</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="8">
@@ -824,7 +820,7 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="9">
@@ -849,7 +845,7 @@
         </is>
       </c>
       <c r="E9" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="10">
@@ -874,7 +870,7 @@
         </is>
       </c>
       <c r="E10" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="11">
@@ -895,11 +891,11 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>L2</t>
+          <t>L1</t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="12">
@@ -920,11 +916,11 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>L1</t>
+          <t>L2</t>
         </is>
       </c>
       <c r="E12" t="n">
-        <v>12</v>
+        <v>7</v>
       </c>
     </row>
     <row r="13">
@@ -945,11 +941,11 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>L2</t>
+          <t>L1</t>
         </is>
       </c>
       <c r="E13" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
     </row>
     <row r="14">
@@ -970,7 +966,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>L2</t>
+          <t>L1</t>
         </is>
       </c>
       <c r="E14" t="n">
@@ -999,7 +995,7 @@
         </is>
       </c>
       <c r="E15" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
     </row>
     <row r="16">
@@ -1020,11 +1016,11 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>L2</t>
+          <t>L1</t>
         </is>
       </c>
       <c r="E16" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="17">
@@ -1049,7 +1045,7 @@
         </is>
       </c>
       <c r="E17" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="18">
@@ -1074,7 +1070,7 @@
         </is>
       </c>
       <c r="E18" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="19">
@@ -1099,7 +1095,7 @@
         </is>
       </c>
       <c r="E19" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="20">
@@ -1120,11 +1116,11 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>L1</t>
+          <t>L2</t>
         </is>
       </c>
       <c r="E20" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="21">
@@ -1145,11 +1141,11 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>L1</t>
+          <t>L2</t>
         </is>
       </c>
       <c r="E21" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="22">
@@ -1160,7 +1156,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1174,7 +1170,7 @@
         </is>
       </c>
       <c r="E22" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
     </row>
     <row r="23">
@@ -1199,7 +1195,7 @@
         </is>
       </c>
       <c r="E23" t="n">
-        <v>4</v>
+        <v>12</v>
       </c>
     </row>
     <row r="24">
@@ -1210,7 +1206,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>P3</t>
+          <t>P4</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1224,7 +1220,7 @@
         </is>
       </c>
       <c r="E24" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
     </row>
     <row r="25">
@@ -1249,7 +1245,7 @@
         </is>
       </c>
       <c r="E25" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
     </row>
     <row r="26">
@@ -1260,7 +1256,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>P4</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1274,7 +1270,7 @@
         </is>
       </c>
       <c r="E26" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
     </row>
     <row r="27">
@@ -1285,7 +1281,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>P3</t>
+          <t>P4</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1299,7 +1295,7 @@
         </is>
       </c>
       <c r="E27" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>